<commit_message>
feat(colab): create a demo to google colab
</commit_message>
<xml_diff>
--- a/output/results.xlsx
+++ b/output/results.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="94" uniqueCount="55">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="86" uniqueCount="50">
   <si>
     <t>SKU_Origen</t>
   </si>
@@ -64,9 +64,6 @@
     <t>Montable   Push  Car Adventure Boy</t>
   </si>
   <si>
-    <t>Carrito De Paseo Push Car Prinsel Adventure Rojo</t>
-  </si>
-  <si>
     <t>Juguete Casita Playhouse Prinsel 2 En 1 Unisex Luz Y Sonidos</t>
   </si>
   <si>
@@ -94,9 +91,6 @@
     <t>2,355.00</t>
   </si>
   <si>
-    <t>1,871.00</t>
-  </si>
-  <si>
     <t>2,879.00</t>
   </si>
   <si>
@@ -115,9 +109,6 @@
     <t>2,499.00</t>
   </si>
   <si>
-    <t>1,970.00</t>
-  </si>
-  <si>
     <t>3,199.00</t>
   </si>
   <si>
@@ -136,46 +127,40 @@
     <t>33%</t>
   </si>
   <si>
-    <t>5%</t>
-  </si>
-  <si>
     <t>10%</t>
   </si>
   <si>
     <t>20%</t>
   </si>
   <si>
-    <t>https://www.mercadolibre.com.mx/montable-push-car-prinsel-adventure-rosa/p/MLM23448401?searchVariation=MLM23448401#polycard_client=search-nordic&amp;searchVariation=MLM23448401&amp;wid=MLM2277931636&amp;position=8&amp;search_layout=grid&amp;type=product&amp;tracking_id=b13790ec-7482-4a02-812e-86d3c6282cb7&amp;sid=search</t>
-  </si>
-  <si>
-    <t>https://www.mercadolibre.com.mx/montable-push-car-prinsel-adventure-rojo/p/MLM23448405?searchVariation=MLM23448405#polycard_client=search-nordic&amp;searchVariation=MLM23448405&amp;wid=MLM2987283252&amp;position=7&amp;search_layout=grid&amp;type=product&amp;tracking_id=b13790ec-7482-4a02-812e-86d3c6282cb7&amp;sid=search</t>
-  </si>
-  <si>
-    <t>https://articulo.mercadolibre.com.mx/MLM-819186928-montable-push-car-prinsel-adventure-rojo-_JM?searchVariation=85393820023#polycard_client=search-nordic&amp;searchVariation=85393820023&amp;position=13&amp;search_layout=grid&amp;type=item&amp;tracking_id=b13790ec-7482-4a02-812e-86d3c6282cb7</t>
-  </si>
-  <si>
-    <t>https://articulo.mercadolibre.com.mx/MLM-3482653740-carro-montable-para-nino-push-car-adventure-sombrilla-rojo-_JM#polycard_client=search-nordic&amp;position=14&amp;search_layout=grid&amp;type=item&amp;tracking_id=b13790ec-7482-4a02-812e-86d3c6282cb7&amp;wid=MLM3482653740&amp;sid=search</t>
-  </si>
-  <si>
-    <t>https://articulo.mercadolibre.com.mx/MLM-1371665566-montable-push-car-adventure-boy-_JM?searchVariation=174143643187#polycard_client=search-nordic&amp;searchVariation=174143643187&amp;position=17&amp;search_layout=grid&amp;type=item&amp;tracking_id=b13790ec-7482-4a02-812e-86d3c6282cb7</t>
-  </si>
-  <si>
-    <t>https://articulo.mercadolibre.com.mx/MLM-1365895208-carrito-de-paseo-push-car-prinsel-adventure-rojo-_JM?searchVariation=174099589239#polycard_client=search-nordic&amp;searchVariation=174099589239&amp;position=18&amp;search_layout=grid&amp;type=item&amp;tracking_id=b13790ec-7482-4a02-812e-86d3c6282cb7</t>
-  </si>
-  <si>
-    <t>https://articulo.mercadolibre.com.mx/MLM-3357610946-juguete-casita-playhouse-prinsel-2-en-1-unisex-luz-y-sonidos-_JM?searchVariation=184799348247#polycard_client=search-nordic&amp;searchVariation=184799348247&amp;position=19&amp;search_layout=grid&amp;type=item&amp;tracking_id=d64448d1-d450-4347-bdbb-a92a157f53b5</t>
-  </si>
-  <si>
-    <t>https://articulo.mercadolibre.com.mx/MLM-2232514817-prinsel-playhouse-2-en-1-unisex-_JM#polycard_client=search-nordic&amp;position=20&amp;search_layout=grid&amp;type=item&amp;tracking_id=d64448d1-d450-4347-bdbb-a92a157f53b5&amp;wid=MLM2232514817&amp;sid=search</t>
-  </si>
-  <si>
-    <t>https://www.mercadolibre.com.mx/playhouse-2-en-1-prinsel-unisex/up/MLMU1137555740#polycard_client=search-nordic&amp;searchVariation=MLMU1137555740&amp;wid=MLM2142108787&amp;position=1&amp;search_layout=grid&amp;type=product&amp;tracking_id=d64448d1-d450-4347-bdbb-a92a157f53b5&amp;sid=search</t>
-  </si>
-  <si>
-    <t>https://www.mercadolibre.com.mx/baby-colecho-prinsel-beige/p/MLM27409971?searchVariation=MLM27409971#polycard_client=search-nordic&amp;searchVariation=MLM27409971&amp;backend_model=search-backend&amp;wid=MLM1999130873&amp;position=2&amp;search_layout=grid&amp;type=product&amp;tracking_id=d6d3571c-0715-4860-aab5-913e30f10739&amp;sid=search</t>
-  </si>
-  <si>
-    <t>https://click1.mercadolibre.com.mx/mclics/clicks/external/MLM/count?a=M1pqzNAq%2Fe3DlyBAsBX4%2Bk4qnyXXpG%2BOhZfCOc4CmkxFQjrPODDKZ0%2BlRbwS2v1wSDjrQwkNEt%2F5edVrWU%2BdySrTY5lAuoLH7Pmrvpov7a6b%2FVkeX1X4wyGM3VLz6%2FHKtLyhqAPjQ7NCKOb9lRqZfoClAt6m65Qg1Ib8Ijepz6Mn0AZ%2Fi5WiFOwKVDy61tbeIIB%2BeI3pEO5NGlL4XEah6eLkksQkMBk8COHcnUzdICb4Vjnv5oZxcViQ9TWwA6hJpV4cy6SBl2iAy43Lx3%2F7wvXjShS6m40N9BRXS4KuvzxnvoY9IE8rMvHskM7%2Fc2JuGZb8MS%2BdEo0ADsJIhLtSCWD1jtWMuT0Ei1DxDh65p9S7vZhDGes3K1E7Oi1aLrKziwtf3fGYoluqd5njS3QiMluD2i5UrdUtsniehsK0cvdVeKdKDRr6JCXCDHbz4I%2BhMVuQImmDbcaiXALVGZKs1ojR0tMRgnfK5OiPza%2B7yFnlS0GeM1TgbF5tOiH3pMNQvYiUUamifMx%2BsSBHcDfpUkZUCKLjEYvOZ8piTP6Oi9ysIcRGowV6HCU%2BRfiV5PQ%2BYqbN7lfwBdjJ6ATH8FCi8oOUYSCX8RMtjTCQebG%2BqjG5%2FoPLMyZcUsVvLNGTb2ytCWFsZYqVYVD5KtDzibK%2FvNABb1%2B8yNEP5GXk5DEufMgQOLX5LwcZbUeiMQjkyIa0MUxskp2NwDQCVAKpNfAdyQiPdoHJlVVsPQ%2F1zq2%2FURl%2BGDQ8KWK5xRodn%2FXUER%2FnxhMkL3qB3D52YvF%2B86rtHoFK4iwNLCyt%2B4gEeEakmAq6JeRVaruKSVOEJnUlxYe%2F%2Fv9pIQxMxQnBfjkcjKRy2kUL8YU2IwHjrEVvjpxibu2mkuIWcGatffNuYbrz8OzvKbdunHvPxFDHgLOgYeOReOwaCXIkc%2FevUxeT3%2BaSS1lgjLhX5AtylantvJXrROucmrgqmg%3D%3D#polycard_client=search-nordic&amp;tracking_id=d6d3571c-0715-4860-aab5-913e30f10739&amp;wid=MLM1999130873&amp;sid=search</t>
+    <t>https://www.mercadolibre.com.mx/montable-push-car-prinsel-adventure-rosa/p/MLM23448401?searchVariation=MLM23448401#polycard_client=search-nordic&amp;searchVariation=MLM23448401&amp;wid=MLM2277931636&amp;position=3&amp;search_layout=grid&amp;type=product&amp;tracking_id=8b2cca1e-345f-4311-9d6e-f8d493cd33ed&amp;sid=search</t>
+  </si>
+  <si>
+    <t>https://www.mercadolibre.com.mx/montable-push-car-prinsel-adventure-rojo/p/MLM23448405?searchVariation=MLM23448405#polycard_client=search-nordic&amp;searchVariation=MLM23448405&amp;wid=MLM2987283252&amp;position=5&amp;search_layout=grid&amp;type=product&amp;tracking_id=8b2cca1e-345f-4311-9d6e-f8d493cd33ed&amp;sid=search</t>
+  </si>
+  <si>
+    <t>https://articulo.mercadolibre.com.mx/MLM-819186928-montable-push-car-prinsel-adventure-rojo-_JM?searchVariation=85393820023#polycard_client=search-nordic&amp;searchVariation=85393820023&amp;position=14&amp;search_layout=grid&amp;type=item&amp;tracking_id=8b2cca1e-345f-4311-9d6e-f8d493cd33ed</t>
+  </si>
+  <si>
+    <t>https://articulo.mercadolibre.com.mx/MLM-3482653740-carro-montable-para-nino-push-car-adventure-sombrilla-rojo-_JM#polycard_client=search-nordic&amp;position=15&amp;search_layout=grid&amp;type=item&amp;tracking_id=8b2cca1e-345f-4311-9d6e-f8d493cd33ed&amp;wid=MLM3482653740&amp;sid=search</t>
+  </si>
+  <si>
+    <t>https://articulo.mercadolibre.com.mx/MLM-1371665566-montable-push-car-adventure-boy-_JM?searchVariation=174143643187#polycard_client=search-nordic&amp;searchVariation=174143643187&amp;position=18&amp;search_layout=grid&amp;type=item&amp;tracking_id=8b2cca1e-345f-4311-9d6e-f8d493cd33ed</t>
+  </si>
+  <si>
+    <t>https://articulo.mercadolibre.com.mx/MLM-3357610946-juguete-casita-playhouse-prinsel-2-en-1-unisex-luz-y-sonidos-_JM?searchVariation=184799348247#polycard_client=search-nordic&amp;searchVariation=184799348247&amp;position=19&amp;search_layout=grid&amp;type=item&amp;tracking_id=9fcb2765-1443-4aa4-bfb4-6070fb7ae3d5</t>
+  </si>
+  <si>
+    <t>https://articulo.mercadolibre.com.mx/MLM-2232514817-prinsel-playhouse-2-en-1-unisex-_JM#polycard_client=search-nordic&amp;position=20&amp;search_layout=grid&amp;type=item&amp;tracking_id=9fcb2765-1443-4aa4-bfb4-6070fb7ae3d5&amp;wid=MLM2232514817&amp;sid=search</t>
+  </si>
+  <si>
+    <t>https://www.mercadolibre.com.mx/playhouse-2-en-1-prinsel-unisex/up/MLMU1137555740#polycard_client=search-nordic&amp;searchVariation=MLMU1137555740&amp;wid=MLM2142108787&amp;position=2&amp;search_layout=grid&amp;type=product&amp;tracking_id=9fcb2765-1443-4aa4-bfb4-6070fb7ae3d5&amp;sid=search</t>
+  </si>
+  <si>
+    <t>https://www.mercadolibre.com.mx/baby-colecho-prinsel-beige/p/MLM27409971?searchVariation=MLM27409971#polycard_client=search-nordic&amp;searchVariation=MLM27409971&amp;backend_model=search-backend&amp;wid=MLM1999130873&amp;position=2&amp;search_layout=grid&amp;type=product&amp;tracking_id=b073fe59-c22c-409f-933c-3813f51a7145&amp;sid=search</t>
+  </si>
+  <si>
+    <t>https://click1.mercadolibre.com.mx/mclics/clicks/external/MLM/count?a=H0PHte6kP2dh%2Br146oLgOpQNnDnMMRYUWiUMxgjfgEyyX9x7P6nCSkDrVg9hNioVsBtwYiVBsUF3UhgkF5JJBHAjwX%2Blt7pLS%2BODuHpWg%2FsPrfVatTQZx8dkeDilI3SSu21YtKNcKbKR%2Fs3eSoEbCezGn4humLuVKDmems%2FJ%2F31VxXqWF5rOGF8xI8dKJut3BNekTHjK5z2DDVEzaSJrMAPKhsXqp5QPUZnLFES3Ti3VkwaGWtH9yvQfDTBem7K0EXnB83XIacAwEbInO2QmM7lLJA0PLWK%2BrJchig5Uw5Y04MdXMQT98eHuUdzySOvU1PQ2%2BA0cvjEMcF04Y4VqoeYZTD3U%2BIvn3hXVY6QA%2BF3Y%2B8yIWazAzmCA4NXMt%2BT8aqFcKaYc8OgWX2bfxPoGdu7%2FJhj7uOdFIH%2FogOyif27huqKsbUDgK92uQrwuQ5XQi6JkL4fgBjaE4K61%2Fl6bCZ2n6J5ZUNk89d%2F11XFSSDPVNstl4%2FlL2zoxObS0w7looPBb4jHo1qMozAzjYZpj7ua1ubsX0%2FnD%2FkCndFYBmrC5z4p7tuIBYkuwcHVXl7inzZvvMo4QPa7nuAP9x9goYqyw6clb9KctrjZyHpyiBPEJYcYzJgzEzBoh08bYZ3Wxxq2jFCYEloq03t%2Br33LgdCOth7iKzS4pbmzHTvxxSfBO6ahsmpCfbzvLnKvoDXcv5F70YF1jtI6J6AZZKXsOGPbixnxRD0cRB%2FzEqSA2X8bkXwlbD9oaI%2Bbwt4ovEPGdZgiDGTIQo51xqNsq1dqOthA%2Bwqn9uZAXYhG0BO%2B2FHmtyegaZTaNjg7gnwOqcHRVmZWOoUrmraMYSm0vnvyPjL8MbAgpv48HDlHOrUgD76xSc6riYK%2BWlYfvxcPLaCSiG9WJtUTn7isXkHaqJISXAL8lAVOL8Uehu5vSpCOFbVjmZXtLksFpOPN1J%2FCcg1O0NBgcDg%3D%3D#polycard_client=search-nordic&amp;tracking_id=b073fe59-c22c-409f-933c-3813f51a7145&amp;wid=MLM1999130873&amp;sid=search</t>
   </si>
   <si>
     <t>mercadolibre</t>
@@ -553,7 +538,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:I12"/>
+  <dimension ref="A1:I11"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="3" max="4" width="12.7109375" style="1" customWidth="1"/>
@@ -596,22 +581,22 @@
         <v>12</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="D2" s="1" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="E2" t="s">
-        <v>37</v>
+        <v>34</v>
       </c>
       <c r="F2" s="3" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="G2" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="H2" s="3" t="s">
-        <v>43</v>
+        <v>39</v>
       </c>
       <c r="I2">
         <v>0.32</v>
@@ -625,22 +610,22 @@
         <v>13</v>
       </c>
       <c r="C3" s="1" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D3" s="1" t="s">
-        <v>32</v>
+        <v>30</v>
       </c>
       <c r="E3" t="s">
-        <v>38</v>
+        <v>35</v>
       </c>
       <c r="F3" s="3" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="G3" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="H3" s="3" t="s">
-        <v>44</v>
+        <v>40</v>
       </c>
       <c r="I3">
         <v>0.66</v>
@@ -654,22 +639,22 @@
         <v>13</v>
       </c>
       <c r="C4" s="1" t="s">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="D4" s="1" t="s">
-        <v>31</v>
+        <v>29</v>
       </c>
       <c r="E4" t="s">
-        <v>39</v>
+        <v>36</v>
       </c>
       <c r="F4" s="3" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="G4" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="H4" s="3" t="s">
-        <v>45</v>
+        <v>41</v>
       </c>
       <c r="I4">
         <v>0.66</v>
@@ -683,19 +668,19 @@
         <v>14</v>
       </c>
       <c r="C5" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="D5" s="1" t="s">
-        <v>24</v>
+        <v>23</v>
       </c>
       <c r="F5" s="3" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="G5" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="H5" s="3" t="s">
-        <v>46</v>
+        <v>42</v>
       </c>
       <c r="I5">
         <v>0.24</v>
@@ -709,19 +694,19 @@
         <v>15</v>
       </c>
       <c r="C6" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="D6" s="1" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
       <c r="F6" s="3" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="G6" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="H6" s="3" t="s">
-        <v>47</v>
+        <v>43</v>
       </c>
       <c r="I6">
         <v>0.26</v>
@@ -729,31 +714,31 @@
     </row>
     <row r="7" spans="1:9">
       <c r="A7" t="s">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="B7" t="s">
         <v>16</v>
       </c>
       <c r="C7" s="1" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="D7" s="1" t="s">
-        <v>33</v>
+        <v>31</v>
       </c>
       <c r="E7" t="s">
-        <v>40</v>
+        <v>37</v>
       </c>
       <c r="F7" s="3" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="G7" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="H7" s="3" t="s">
-        <v>48</v>
+        <v>44</v>
       </c>
       <c r="I7">
-        <v>0.32</v>
+        <v>0.26</v>
       </c>
     </row>
     <row r="8" spans="1:9">
@@ -764,25 +749,22 @@
         <v>17</v>
       </c>
       <c r="C8" s="1" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="D8" s="1" t="s">
-        <v>34</v>
-      </c>
-      <c r="E8" t="s">
-        <v>41</v>
+        <v>26</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="G8" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="H8" s="3" t="s">
-        <v>49</v>
+        <v>45</v>
       </c>
       <c r="I8">
-        <v>0.26</v>
+        <v>0.35</v>
       </c>
     </row>
     <row r="9" spans="1:9">
@@ -793,19 +775,22 @@
         <v>18</v>
       </c>
       <c r="C9" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="D9" s="1" t="s">
-        <v>28</v>
+        <v>32</v>
+      </c>
+      <c r="E9" t="s">
+        <v>38</v>
       </c>
       <c r="F9" s="3" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="G9" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="H9" s="3" t="s">
-        <v>50</v>
+        <v>46</v>
       </c>
       <c r="I9">
         <v>0.35</v>
@@ -813,31 +798,31 @@
     </row>
     <row r="10" spans="1:9">
       <c r="A10" t="s">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="B10" t="s">
         <v>19</v>
       </c>
       <c r="C10" s="1" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="D10" s="1" t="s">
-        <v>35</v>
+        <v>33</v>
       </c>
       <c r="E10" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="F10" s="3" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="G10" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="H10" s="3" t="s">
-        <v>51</v>
+        <v>47</v>
       </c>
       <c r="I10">
-        <v>0.35</v>
+        <v>0.24</v>
       </c>
     </row>
     <row r="11" spans="1:9">
@@ -845,83 +830,52 @@
         <v>11</v>
       </c>
       <c r="B11" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
       <c r="C11" s="1" t="s">
-        <v>30</v>
+        <v>28</v>
       </c>
       <c r="D11" s="1" t="s">
-        <v>36</v>
+        <v>33</v>
       </c>
       <c r="E11" t="s">
-        <v>42</v>
+        <v>38</v>
       </c>
       <c r="F11" s="3" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="G11" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="H11" s="3" t="s">
-        <v>52</v>
+        <v>48</v>
       </c>
       <c r="I11">
         <v>0.24</v>
       </c>
     </row>
-    <row r="12" spans="1:9">
-      <c r="A12" t="s">
-        <v>11</v>
-      </c>
-      <c r="B12" t="s">
-        <v>20</v>
-      </c>
-      <c r="C12" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="D12" s="1" t="s">
-        <v>36</v>
-      </c>
-      <c r="E12" t="s">
-        <v>42</v>
-      </c>
-      <c r="F12" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="G12" t="s">
-        <v>54</v>
-      </c>
-      <c r="H12" s="3" t="s">
-        <v>53</v>
-      </c>
-      <c r="I12">
-        <v>0.24</v>
-      </c>
-    </row>
   </sheetData>
   <hyperlinks>
-    <hyperlink ref="F2" r:id="rId1" location="polycard_client=search-nordic&amp;searchVariation=MLM23448401&amp;wid=MLM2277931636&amp;position=8&amp;search_layout=grid&amp;type=product&amp;tracking_id=b13790ec-7482-4a02-812e-86d3c6282cb7&amp;sid=search"/>
-    <hyperlink ref="H2" r:id="rId2" location="polycard_client=search-nordic&amp;searchVariation=MLM23448401&amp;wid=MLM2277931636&amp;position=8&amp;search_layout=grid&amp;type=product&amp;tracking_id=b13790ec-7482-4a02-812e-86d3c6282cb7&amp;sid=search"/>
-    <hyperlink ref="F3" r:id="rId3" location="polycard_client=search-nordic&amp;searchVariation=MLM23448405&amp;wid=MLM2987283252&amp;position=7&amp;search_layout=grid&amp;type=product&amp;tracking_id=b13790ec-7482-4a02-812e-86d3c6282cb7&amp;sid=search"/>
-    <hyperlink ref="H3" r:id="rId4" location="polycard_client=search-nordic&amp;searchVariation=MLM23448405&amp;wid=MLM2987283252&amp;position=7&amp;search_layout=grid&amp;type=product&amp;tracking_id=b13790ec-7482-4a02-812e-86d3c6282cb7&amp;sid=search"/>
-    <hyperlink ref="F4" r:id="rId5" location="polycard_client=search-nordic&amp;searchVariation=85393820023&amp;position=13&amp;search_layout=grid&amp;type=item&amp;tracking_id=b13790ec-7482-4a02-812e-86d3c6282cb7"/>
-    <hyperlink ref="H4" r:id="rId6" location="polycard_client=search-nordic&amp;searchVariation=85393820023&amp;position=13&amp;search_layout=grid&amp;type=item&amp;tracking_id=b13790ec-7482-4a02-812e-86d3c6282cb7"/>
-    <hyperlink ref="F5" r:id="rId7" location="polycard_client=search-nordic&amp;position=14&amp;search_layout=grid&amp;type=item&amp;tracking_id=b13790ec-7482-4a02-812e-86d3c6282cb7&amp;wid=MLM3482653740&amp;sid=search"/>
-    <hyperlink ref="H5" r:id="rId8" location="polycard_client=search-nordic&amp;position=14&amp;search_layout=grid&amp;type=item&amp;tracking_id=b13790ec-7482-4a02-812e-86d3c6282cb7&amp;wid=MLM3482653740&amp;sid=search"/>
-    <hyperlink ref="F6" r:id="rId9" location="polycard_client=search-nordic&amp;searchVariation=174143643187&amp;position=17&amp;search_layout=grid&amp;type=item&amp;tracking_id=b13790ec-7482-4a02-812e-86d3c6282cb7"/>
-    <hyperlink ref="H6" r:id="rId10" location="polycard_client=search-nordic&amp;searchVariation=174143643187&amp;position=17&amp;search_layout=grid&amp;type=item&amp;tracking_id=b13790ec-7482-4a02-812e-86d3c6282cb7"/>
-    <hyperlink ref="F7" r:id="rId11" location="polycard_client=search-nordic&amp;searchVariation=174099589239&amp;position=18&amp;search_layout=grid&amp;type=item&amp;tracking_id=b13790ec-7482-4a02-812e-86d3c6282cb7"/>
-    <hyperlink ref="H7" r:id="rId12" location="polycard_client=search-nordic&amp;searchVariation=174099589239&amp;position=18&amp;search_layout=grid&amp;type=item&amp;tracking_id=b13790ec-7482-4a02-812e-86d3c6282cb7"/>
-    <hyperlink ref="F8" r:id="rId13" location="polycard_client=search-nordic&amp;searchVariation=184799348247&amp;position=19&amp;search_layout=grid&amp;type=item&amp;tracking_id=d64448d1-d450-4347-bdbb-a92a157f53b5"/>
-    <hyperlink ref="H8" r:id="rId14" location="polycard_client=search-nordic&amp;searchVariation=184799348247&amp;position=19&amp;search_layout=grid&amp;type=item&amp;tracking_id=d64448d1-d450-4347-bdbb-a92a157f53b5"/>
-    <hyperlink ref="F9" r:id="rId15" location="polycard_client=search-nordic&amp;position=20&amp;search_layout=grid&amp;type=item&amp;tracking_id=d64448d1-d450-4347-bdbb-a92a157f53b5&amp;wid=MLM2232514817&amp;sid=search"/>
-    <hyperlink ref="H9" r:id="rId16" location="polycard_client=search-nordic&amp;position=20&amp;search_layout=grid&amp;type=item&amp;tracking_id=d64448d1-d450-4347-bdbb-a92a157f53b5&amp;wid=MLM2232514817&amp;sid=search"/>
-    <hyperlink ref="F10" r:id="rId17" location="polycard_client=search-nordic&amp;searchVariation=MLMU1137555740&amp;wid=MLM2142108787&amp;position=1&amp;search_layout=grid&amp;type=product&amp;tracking_id=d64448d1-d450-4347-bdbb-a92a157f53b5&amp;sid=search"/>
-    <hyperlink ref="H10" r:id="rId18" location="polycard_client=search-nordic&amp;searchVariation=MLMU1137555740&amp;wid=MLM2142108787&amp;position=1&amp;search_layout=grid&amp;type=product&amp;tracking_id=d64448d1-d450-4347-bdbb-a92a157f53b5&amp;sid=search"/>
-    <hyperlink ref="F11" r:id="rId19" location="polycard_client=search-nordic&amp;searchVariation=MLM27409971&amp;backend_model=search-backend&amp;wid=MLM1999130873&amp;position=2&amp;search_layout=grid&amp;type=product&amp;tracking_id=d6d3571c-0715-4860-aab5-913e30f10739&amp;sid=search"/>
-    <hyperlink ref="H11" r:id="rId20" location="polycard_client=search-nordic&amp;searchVariation=MLM27409971&amp;backend_model=search-backend&amp;wid=MLM1999130873&amp;position=2&amp;search_layout=grid&amp;type=product&amp;tracking_id=d6d3571c-0715-4860-aab5-913e30f10739&amp;sid=search"/>
-    <hyperlink ref="F12" r:id="rId21" location="polycard_client=search-nordic&amp;tracking_id=d6d3571c-0715-4860-aab5-913e30f10739&amp;wid=MLM1999130873&amp;sid=search"/>
-    <hyperlink ref="H12" r:id="rId22" location="polycard_client=search-nordic&amp;tracking_id=d6d3571c-0715-4860-aab5-913e30f10739&amp;wid=MLM1999130873&amp;sid=search"/>
+    <hyperlink ref="F2" r:id="rId1" location="polycard_client=search-nordic&amp;searchVariation=MLM23448401&amp;wid=MLM2277931636&amp;position=3&amp;search_layout=grid&amp;type=product&amp;tracking_id=8b2cca1e-345f-4311-9d6e-f8d493cd33ed&amp;sid=search"/>
+    <hyperlink ref="H2" r:id="rId2" location="polycard_client=search-nordic&amp;searchVariation=MLM23448401&amp;wid=MLM2277931636&amp;position=3&amp;search_layout=grid&amp;type=product&amp;tracking_id=8b2cca1e-345f-4311-9d6e-f8d493cd33ed&amp;sid=search"/>
+    <hyperlink ref="F3" r:id="rId3" location="polycard_client=search-nordic&amp;searchVariation=MLM23448405&amp;wid=MLM2987283252&amp;position=5&amp;search_layout=grid&amp;type=product&amp;tracking_id=8b2cca1e-345f-4311-9d6e-f8d493cd33ed&amp;sid=search"/>
+    <hyperlink ref="H3" r:id="rId4" location="polycard_client=search-nordic&amp;searchVariation=MLM23448405&amp;wid=MLM2987283252&amp;position=5&amp;search_layout=grid&amp;type=product&amp;tracking_id=8b2cca1e-345f-4311-9d6e-f8d493cd33ed&amp;sid=search"/>
+    <hyperlink ref="F4" r:id="rId5" location="polycard_client=search-nordic&amp;searchVariation=85393820023&amp;position=14&amp;search_layout=grid&amp;type=item&amp;tracking_id=8b2cca1e-345f-4311-9d6e-f8d493cd33ed"/>
+    <hyperlink ref="H4" r:id="rId6" location="polycard_client=search-nordic&amp;searchVariation=85393820023&amp;position=14&amp;search_layout=grid&amp;type=item&amp;tracking_id=8b2cca1e-345f-4311-9d6e-f8d493cd33ed"/>
+    <hyperlink ref="F5" r:id="rId7" location="polycard_client=search-nordic&amp;position=15&amp;search_layout=grid&amp;type=item&amp;tracking_id=8b2cca1e-345f-4311-9d6e-f8d493cd33ed&amp;wid=MLM3482653740&amp;sid=search"/>
+    <hyperlink ref="H5" r:id="rId8" location="polycard_client=search-nordic&amp;position=15&amp;search_layout=grid&amp;type=item&amp;tracking_id=8b2cca1e-345f-4311-9d6e-f8d493cd33ed&amp;wid=MLM3482653740&amp;sid=search"/>
+    <hyperlink ref="F6" r:id="rId9" location="polycard_client=search-nordic&amp;searchVariation=174143643187&amp;position=18&amp;search_layout=grid&amp;type=item&amp;tracking_id=8b2cca1e-345f-4311-9d6e-f8d493cd33ed"/>
+    <hyperlink ref="H6" r:id="rId10" location="polycard_client=search-nordic&amp;searchVariation=174143643187&amp;position=18&amp;search_layout=grid&amp;type=item&amp;tracking_id=8b2cca1e-345f-4311-9d6e-f8d493cd33ed"/>
+    <hyperlink ref="F7" r:id="rId11" location="polycard_client=search-nordic&amp;searchVariation=184799348247&amp;position=19&amp;search_layout=grid&amp;type=item&amp;tracking_id=9fcb2765-1443-4aa4-bfb4-6070fb7ae3d5"/>
+    <hyperlink ref="H7" r:id="rId12" location="polycard_client=search-nordic&amp;searchVariation=184799348247&amp;position=19&amp;search_layout=grid&amp;type=item&amp;tracking_id=9fcb2765-1443-4aa4-bfb4-6070fb7ae3d5"/>
+    <hyperlink ref="F8" r:id="rId13" location="polycard_client=search-nordic&amp;position=20&amp;search_layout=grid&amp;type=item&amp;tracking_id=9fcb2765-1443-4aa4-bfb4-6070fb7ae3d5&amp;wid=MLM2232514817&amp;sid=search"/>
+    <hyperlink ref="H8" r:id="rId14" location="polycard_client=search-nordic&amp;position=20&amp;search_layout=grid&amp;type=item&amp;tracking_id=9fcb2765-1443-4aa4-bfb4-6070fb7ae3d5&amp;wid=MLM2232514817&amp;sid=search"/>
+    <hyperlink ref="F9" r:id="rId15" location="polycard_client=search-nordic&amp;searchVariation=MLMU1137555740&amp;wid=MLM2142108787&amp;position=2&amp;search_layout=grid&amp;type=product&amp;tracking_id=9fcb2765-1443-4aa4-bfb4-6070fb7ae3d5&amp;sid=search"/>
+    <hyperlink ref="H9" r:id="rId16" location="polycard_client=search-nordic&amp;searchVariation=MLMU1137555740&amp;wid=MLM2142108787&amp;position=2&amp;search_layout=grid&amp;type=product&amp;tracking_id=9fcb2765-1443-4aa4-bfb4-6070fb7ae3d5&amp;sid=search"/>
+    <hyperlink ref="F10" r:id="rId17" location="polycard_client=search-nordic&amp;searchVariation=MLM27409971&amp;backend_model=search-backend&amp;wid=MLM1999130873&amp;position=2&amp;search_layout=grid&amp;type=product&amp;tracking_id=b073fe59-c22c-409f-933c-3813f51a7145&amp;sid=search"/>
+    <hyperlink ref="H10" r:id="rId18" location="polycard_client=search-nordic&amp;searchVariation=MLM27409971&amp;backend_model=search-backend&amp;wid=MLM1999130873&amp;position=2&amp;search_layout=grid&amp;type=product&amp;tracking_id=b073fe59-c22c-409f-933c-3813f51a7145&amp;sid=search"/>
+    <hyperlink ref="F11" r:id="rId19" location="polycard_client=search-nordic&amp;tracking_id=b073fe59-c22c-409f-933c-3813f51a7145&amp;wid=MLM1999130873&amp;sid=search"/>
+    <hyperlink ref="H11" r:id="rId20" location="polycard_client=search-nordic&amp;tracking_id=b073fe59-c22c-409f-933c-3813f51a7145&amp;wid=MLM1999130873&amp;sid=search"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>